<commit_message>
TSV canonici, XLSX derivati con make xlsx (T-80, D-015)
Nuovo tools/tsv_to_xlsx.py: giro TSV -> XLSX -> TSV verificato byte
per byte sui sette fogli. xlsx_to_tsv.py resta per riportare nei TSV
una modifica fatta in Excel. Dati invariati: 16.045 / 17.203 triple.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/LiteraryWorks.xlsx
+++ b/data/source/xlsx/LiteraryWorks.xlsx
@@ -1,94 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lorenzo.sabatino3\Desktop\Atlante Gadda_step\GaddAtlas_ontology\NEW_DB\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD84FE94-D13F-4200-876B-E12DF6609EF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="LiteraryWorks" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LiteraryWorks" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
-  <si>
-    <t>Work_ID</t>
-  </si>
-  <si>
-    <t>Full_Title</t>
-  </si>
-  <si>
-    <t>Author</t>
-  </si>
-  <si>
-    <t>Publication_Year</t>
-  </si>
-  <si>
-    <t>Edition_Used</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>quer_pasticciaccio</t>
-  </si>
-  <si>
-    <t>Quer pasticciaccio brutto de via Merulana</t>
-  </si>
-  <si>
-    <t>Carlo Emilio Gadda</t>
-  </si>
-  <si>
-    <t>Garzanti, Milano, 1957 (ed. definitiva)</t>
-  </si>
-  <si>
-    <t>Romanzo giallo-filosofico; prima pubblicazione parziale su Letteratura (1946), edizione in volume 1957.</t>
-  </si>
-  <si>
-    <t>quer_pasticciaccio_letteratura</t>
-  </si>
-  <si>
-    <t>Letteratura, Bonsanti</t>
-  </si>
-  <si>
-    <t>quer_pasticciaccio_adelphi</t>
-  </si>
-  <si>
-    <t>Adelphi</t>
-  </si>
-  <si>
-    <t>Ripubblicazione curata da Giorgio Pinotti</t>
-  </si>
-  <si>
-    <t>Prima pubblicazione in 5 tratti sulla rivista Letteratura, dal 1946 al 1948</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -106,23 +46,81 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normale" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -410,96 +408,134 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="35.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="31.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="86.21875" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Work_ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Full_Title</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Author</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Publication_Year</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Edition_Used</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="1">
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>quer_pasticciaccio</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Quer pasticciaccio brutto de via Merulana</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Carlo Emilio Gadda</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
         <v>1957</v>
       </c>
-      <c r="E2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" t="s">
-        <v>10</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Garzanti, Milano, 1957 (ed. definitiva)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Romanzo giallo-filosofico; prima pubblicazione parziale su Letteratura (1946), edizione in volume 1957.</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>quer_pasticciaccio_letteratura</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Quer pasticciaccio brutto de via Merulana</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Carlo Emilio Gadda</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
         <v>1946</v>
       </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" t="s">
-        <v>16</v>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Letteratura, Bonsanti</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Prima pubblicazione in 5 tratti sulla rivista Letteratura, dal 1946 al 1948</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>quer_pasticciaccio_adelphi</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Quer pasticciaccio brutto de via Merulana</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Carlo Emilio Gadda</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
         <v>2018</v>
       </c>
-      <c r="E4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" t="s">
-        <v>15</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Adelphi</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Ripubblicazione curata da Giorgio Pinotti</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
opera e testimoni: modello minimo, sei testimoni (T-40, D-052)
chora:Witness con tipo, data, curatore, sede; QPL, dtsFG, bzFG, QP57,
RR II, QP (riferimento). prov:wasDerivedFrom solo dove documentato
(QP57 <- QPL, bzFG). Allineamento LRMoo dichiarato nel mapping. Il palazzo
degli ori come opera correlata. Shape 14.
TBox 1.070 -> 1.146, ABox 26.249 -> 26.300, SHACL conforme.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/xlsx/LiteraryWorks.xlsx
+++ b/data/source/xlsx/LiteraryWorks.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,6 +447,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Related_Work</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -467,14 +472,9 @@
       <c r="D2" t="n">
         <v>1957</v>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Garzanti, Milano, 1957 (ed. definitiva)</t>
-        </is>
-      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Romanzo giallo-filosofico; prima pubblicazione parziale su Letteratura (1946), edizione in volume 1957.</t>
+          <t>Romanzo. Testimoni in Witnesses.tsv (D-052): QPL, dtsFG, bzFG, QP57, RR II, QP (testo di riferimento).</t>
         </is>
       </c>
     </row>
@@ -535,6 +535,36 @@
       <c r="F4" t="inlineStr">
         <is>
           <t>Ripubblicazione curata da Giorgio Pinotti</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>il_palazzo_degli_ori</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Il palazzo degli ori</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Carlo Emilio Gadda</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1948</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Soggetto cinematografico scritto nel 1948 per la Lux Film, con la «sceneggiatura minore» La casa dei ricchi: derivazione per un altro medium (Pinotti 2016, pp. 201–203). Opera correlata, senza occorrenze, fuori dall'interfaccia (DM-04).</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>quer_pasticciaccio</t>
         </is>
       </c>
     </row>

</xml_diff>